<commit_message>
feat:optimize the display page and parsing logic
</commit_message>
<xml_diff>
--- a/demo_reports.xlsx
+++ b/demo_reports.xlsx
@@ -451,82 +451,82 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>djxh</t>
+          <t>报告编号</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>shxydm</t>
+          <t>统一社会信用代码</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>nsrmc</t>
+          <t>纳税人名称</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>fxrwmc</t>
+          <t>风险任务名称</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>rwcjrq</t>
+          <t>任务创建日期</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>rwwcsj</t>
+          <t>任务完成时间</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ydxx</t>
+          <t>疑点信息</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>sfywt</t>
+          <t>人工判断</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ydry</t>
+          <t>应对人员</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>qksm</t>
+          <t>情况说明</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>sbgzqk</t>
+          <t>申报更正情况</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>rkhj</t>
+          <t>入库合计</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>zgswjgdm</t>
+          <t>主管税务机关代码</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>zgswskfjmc</t>
+          <t>主管税务所科分局名称</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>rdfxnsr</t>
+          <t>认定风险纳税人</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>biztime</t>
+          <t>业务时间</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>增值税进项税额异常增长风险核查</t>
+          <t>2026年06月增值税管理条线第01批上海市税务局第01批软件和信息技术服务行业风险任务</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>无问题</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>销售收入波动及毛利率偏低风险核查</t>
+          <t>2026年06月企业所得税管理条线第01批上海市税务局第02批批发零售行业风险任务</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>有问题</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>成本费用率异常风险核查</t>
+          <t>2026年06月企业所得税管理条线第02批上海市税务局第01批设备服务行业风险任务</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>无法判断</t>
+          <t>有问题</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>发票开具金额与申报收入差异风险核查</t>
+          <t>2026年06月增值税管理条线第02批上海市税务局第01批餐饮服务行业风险任务</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>有问题</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>运输服务进项抵扣真实性风险核查</t>
+          <t>2026年06月增值税管理条线第03批上海市税务局第01批交通运输行业风险任务</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>部分存在问题</t>
+          <t>有问题</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat:optimize 'sfywt' display text,add 'abstract' at the top of the result of reviewing
</commit_message>
<xml_diff>
--- a/demo_reports.xlsx
+++ b/demo_reports.xlsx
@@ -451,82 +451,82 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>报告编号</t>
+          <t>djxh</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>统一社会信用代码</t>
+          <t>shxydm</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>纳税人名称</t>
+          <t>nsrmc</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>风险任务名称</t>
+          <t>fxrwmc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>任务创建日期</t>
+          <t>rwcjrq</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>任务完成时间</t>
+          <t>rwwcsj</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>疑点信息</t>
+          <t>ydxx</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>人工判断</t>
+          <t>sfywt</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>应对人员</t>
+          <t>ydry</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>情况说明</t>
+          <t>qksm</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>申报更正情况</t>
+          <t>sbgzqk</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>入库合计</t>
+          <t>rkhj</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>主管税务机关代码</t>
+          <t>zgswjgdm</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>主管税务所科分局名称</t>
+          <t>zgswskfjmc</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>认定风险纳税人</t>
+          <t>rdfxnsr</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>业务时间</t>
+          <t>biztime</t>
         </is>
       </c>
     </row>

</xml_diff>